<commit_message>
scan: seg8 2026-08-14 16:18 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq0_2026-08-14.xlsx
+++ b/output/full_scan/batch_seq0_2026-08-14.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O117"/>
+  <dimension ref="A1:O118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1088,7 +1088,7 @@
         <v>27.22510491877956</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>1.83016245255195</v>
+        <v>1.830162452551949</v>
       </c>
       <c r="K12" s="2" t="n">
         <v>0</v>
@@ -2382,21 +2382,21 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>8289</v>
+        <v>8046</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>泰藝</t>
+          <t>南電</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>404.9635828991812</v>
+        <v>406.2948270361717</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>47.1</v>
+        <v>1305</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2407,13 +2407,13 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>49.84652717542686</v>
+        <v>61.6805191785566</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>25.70756503392619</v>
+        <v>14.71004619914134</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>0.7962968560128386</v>
+        <v>1.852348660304362</v>
       </c>
       <c r="K37" s="2" t="n">
         <v>0</v>
@@ -2425,31 +2425,31 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>1.433343226702728</v>
+        <v>25.69687863150966</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>8249</v>
+        <v>8289</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>菱光</t>
+          <t>泰藝</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v/>
       </c>
       <c r="D38" s="2" t="n">
-        <v>393.6388199029294</v>
+        <v>404.9635828991812</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>42.05</v>
+        <v>47.1</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2460,13 +2460,13 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>41.91934330418641</v>
+        <v>49.84652717542686</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>22.95366002305832</v>
+        <v>25.70756503392619</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>0.8257741821651686</v>
+        <v>0.7962968560128386</v>
       </c>
       <c r="K38" s="2" t="n">
         <v>0</v>
@@ -2478,31 +2478,31 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>0.3615577221280015</v>
+        <v>1.433343226702728</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>8074</v>
+        <v>8249</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>鉅橡</t>
+          <t>菱光</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v/>
       </c>
       <c r="D39" s="2" t="n">
-        <v>391.6650468157066</v>
+        <v>393.6388199029294</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>56.7</v>
+        <v>42.05</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2513,16 +2513,16 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>48.98082872818655</v>
+        <v>41.91934330418641</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>25.77294358534156</v>
+        <v>22.95366002305832</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>0.8441920898040763</v>
+        <v>0.8257741821651686</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L39" s="2" t="n">
         <v>0</v>
@@ -2531,31 +2531,31 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>1.217830451758716</v>
+        <v>0.3615577221280015</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, foreign_buy_3d, adx_trending, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>8227</v>
+        <v>8074</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>巨有科技</t>
+          <t>鉅橡</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>388.9490123544499</v>
+        <v>391.6650468157066</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>151.5</v>
+        <v>56.7</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2566,16 +2566,16 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>46.41103457783559</v>
+        <v>48.98082872818655</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>25.12425384456468</v>
+        <v>25.77294358534156</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>0.6494950167807951</v>
+        <v>0.8441920898040763</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L40" s="2" t="n">
         <v>0</v>
@@ -2584,31 +2584,31 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>3.076780195179208</v>
+        <v>1.217830451758716</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, foreign_buy_3d, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>8215</v>
+        <v>8227</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>明基材</t>
+          <t>巨有科技</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
         <v/>
       </c>
       <c r="D41" s="2" t="n">
-        <v>387.8714124118381</v>
+        <v>388.9490123544499</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>24.6</v>
+        <v>151.5</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2619,13 +2619,13 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>46.56521781184875</v>
+        <v>46.41103457783559</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>27.50295317376576</v>
+        <v>25.12425384456468</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>0.6773384883241953</v>
+        <v>0.6494950167807951</v>
       </c>
       <c r="K41" s="2" t="n">
         <v>0</v>
@@ -2637,31 +2637,31 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>0.3771413771358261</v>
+        <v>3.076780195179208</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>8111</v>
+        <v>8215</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>立碁</t>
+          <t>明基材</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>383.458349724282</v>
+        <v>387.8714124118381</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>55.5</v>
+        <v>24.6</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2672,16 +2672,16 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>46.17465678893983</v>
+        <v>46.56521781184875</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>20.07320514458494</v>
+        <v>27.50295317376576</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>0.2458349724282023</v>
+        <v>0.6773384883241953</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L42" s="2" t="n">
         <v>0</v>
@@ -2690,31 +2690,31 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-0.4458720183205131</v>
+        <v>0.3771413771358261</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>8049</v>
+        <v>8111</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>晶采</t>
+          <t>立碁</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>380.6000097093465</v>
+        <v>383.458349724282</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>26.45</v>
+        <v>55.5</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2725,16 +2725,16 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>53.02689560032901</v>
+        <v>46.17465678893983</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>12.40960404580573</v>
+        <v>20.07320514458494</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>2.995771863322328</v>
+        <v>0.2458349724282023</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L43" s="2" t="n">
         <v>0</v>
@@ -2743,31 +2743,31 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>0.1065698961799115</v>
+        <v>-0.4458720183205131</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>8109</v>
+        <v>8049</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>博大</t>
+          <t>晶采</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>377.8565751029011</v>
+        <v>380.6000097093465</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>131</v>
+        <v>26.45</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2778,13 +2778,13 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>53.12110910292135</v>
+        <v>53.02689560032901</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>15.47916729724443</v>
+        <v>12.40960404580573</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>0.8041192195378226</v>
+        <v>2.995771863322328</v>
       </c>
       <c r="K44" s="2" t="n">
         <v>0</v>
@@ -2796,31 +2796,31 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.6311910561678449</v>
+        <v>0.1065698961799115</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>8088</v>
+        <v>8109</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>品安</t>
+          <t>博大</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>377.669124203492</v>
+        <v>377.8565751029011</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>48.25</v>
+        <v>131</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2831,13 +2831,13 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>46.69028261794819</v>
+        <v>53.12110910292135</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>19.49616842180395</v>
+        <v>15.47916729724443</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>1.024762583901572</v>
+        <v>0.8041192195378226</v>
       </c>
       <c r="K45" s="2" t="n">
         <v>0</v>
@@ -2849,31 +2849,31 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>0.9237926894169596</v>
+        <v>0.6311910561678449</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>8438</v>
+        <v>8088</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>昶昕</t>
+          <t>品安</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>375.5498863802496</v>
+        <v>377.669124203492</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>67.2</v>
+        <v>48.25</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2884,13 +2884,13 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>43.849464145875</v>
+        <v>46.69028261794819</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>26.82968161561736</v>
+        <v>19.49616842180395</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>0.4993172240855711</v>
+        <v>1.024762583901572</v>
       </c>
       <c r="K46" s="2" t="n">
         <v>0</v>
@@ -2902,31 +2902,31 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>1.666555364258926</v>
+        <v>0.9237926894169596</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>8429</v>
+        <v>8438</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>金麗-KY</t>
+          <t>昶昕</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>373.2811189783028</v>
+        <v>375.5498863802496</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>6.04</v>
+        <v>67.2</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2937,13 +2937,13 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>43.5445794373754</v>
+        <v>43.849464145875</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>11.63583474181435</v>
+        <v>26.82968161561736</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0.9370661459833166</v>
+        <v>0.4993172240855711</v>
       </c>
       <c r="K47" s="2" t="n">
         <v>0</v>
@@ -2955,31 +2955,31 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.009568740845229301</v>
+        <v>1.666555364258926</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>8422</v>
+        <v>8429</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>可寧衛*</t>
+          <t>金麗-KY</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>370.1297817644671</v>
+        <v>373.2811189783028</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>26.4</v>
+        <v>6.04</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2990,13 +2990,13 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>49.7428568971933</v>
+        <v>43.5445794373754</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>12.56651633332299</v>
+        <v>11.63583474181435</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>0.4579492514300651</v>
+        <v>0.9370661459833166</v>
       </c>
       <c r="K48" s="2" t="n">
         <v>0</v>
@@ -3008,31 +3008,31 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>0.1708200203979276</v>
+        <v>0.009568740845229301</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>8105</v>
+        <v>8422</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>凌巨</t>
+          <t>可寧衛*</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>368.9444687639827</v>
+        <v>370.1297817644671</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>16.75</v>
+        <v>26.4</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3043,13 +3043,13 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>45.4447473907985</v>
+        <v>49.7428568971933</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>24.14223011975315</v>
+        <v>12.56651633332299</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>0.3882829345696671</v>
+        <v>0.4579492514300651</v>
       </c>
       <c r="K49" s="2" t="n">
         <v>0</v>
@@ -3061,31 +3061,31 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.2293236971945386</v>
+        <v>0.1708200203979276</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>8069</v>
+        <v>8105</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>元太</t>
+          <t>凌巨</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>368.0286079063476</v>
+        <v>368.9444687639827</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>165.5</v>
+        <v>16.75</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3096,13 +3096,13 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>36.43826039427462</v>
+        <v>45.4447473907985</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>13.28002379465443</v>
+        <v>24.14223011975315</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>1.850379003678276</v>
+        <v>0.3882829345696671</v>
       </c>
       <c r="K50" s="2" t="n">
         <v>0</v>
@@ -3114,31 +3114,31 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-2.106834482976662</v>
+        <v>0.2293236971945386</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>9955</v>
+        <v>8069</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>佳龍</t>
+          <t>元太</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>366.7755878028021</v>
+        <v>368.0286079063476</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>24.55</v>
+        <v>165.5</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3149,13 +3149,13 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>50.42718298612665</v>
+        <v>36.43826039427462</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>26.8499237272928</v>
+        <v>13.28002379465443</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0.8389885482105484</v>
+        <v>1.850379003678276</v>
       </c>
       <c r="K51" s="2" t="n">
         <v>0</v>
@@ -3167,31 +3167,31 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.3079111382478636</v>
+        <v>-2.106834482976662</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>8162</v>
+        <v>9955</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>微矽電子-創</t>
+          <t>佳龍</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>366.1575742983319</v>
+        <v>366.7755878028021</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>59.6</v>
+        <v>24.55</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3202,13 +3202,13 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>50.18057822433838</v>
+        <v>50.42718298612665</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>29.82751937662699</v>
+        <v>26.8499237272928</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0.7779123302967276</v>
+        <v>0.8389885482105484</v>
       </c>
       <c r="K52" s="2" t="n">
         <v>0</v>
@@ -3220,31 +3220,31 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>1.431546888995365</v>
+        <v>0.3079111382478636</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>8488</v>
+        <v>8162</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>吉源-KY</t>
+          <t>微矽電子-創</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>359.4820342884808</v>
+        <v>366.1575742983319</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>9.94</v>
+        <v>59.6</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3255,13 +3255,13 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>48.99557921270888</v>
+        <v>50.18057822433838</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>10.07211251307819</v>
+        <v>29.82751937662699</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.0620258647856156</v>
+        <v>0.7779123302967276</v>
       </c>
       <c r="K53" s="2" t="n">
         <v>0</v>
@@ -3273,31 +3273,31 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>-0.0388666628476301</v>
+        <v>1.431546888995365</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>8067</v>
+        <v>8488</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>志旭</t>
+          <t>吉源-KY</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>358.5221934234521</v>
+        <v>359.4820342884808</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>12.5</v>
+        <v>9.94</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>43.29824218850093</v>
+        <v>48.99557921270888</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>8.712179327605412</v>
+        <v>10.07211251307819</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.9651956364678556</v>
+        <v>0.0620258647856156</v>
       </c>
       <c r="K54" s="2" t="n">
         <v>0</v>
@@ -3326,31 +3326,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>-0.0546901818228203</v>
+        <v>-0.0388666628476301</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>8043</v>
+        <v>8067</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>蜜望實</t>
+          <t>志旭</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>357.5350298303215</v>
+        <v>358.5221934234521</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>146</v>
+        <v>12.5</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,16 +3361,16 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>49.85313704191143</v>
+        <v>43.29824218850093</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>19.23875179791283</v>
+        <v>8.712179327605412</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.5567447746452053</v>
+        <v>0.9651956364678556</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L55" s="2" t="n">
         <v>0</v>
@@ -3379,31 +3379,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>3.363051115899847</v>
+        <v>-0.0546901818228203</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>8131</v>
+        <v>8043</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>福懋科</t>
+          <t>蜜望實</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>353.0156864752025</v>
+        <v>357.5350298303215</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>65.2</v>
+        <v>146</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,16 +3414,16 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>49.27097146593565</v>
+        <v>49.85313704191143</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>11.07449581396929</v>
+        <v>19.23875179791283</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>0.8157288007792904</v>
+        <v>0.5567447746452053</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L56" s="2" t="n">
         <v>0</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.7405550201103304</v>
+        <v>3.363051115899847</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>8150</v>
+        <v>8131</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>南茂</t>
+          <t>福懋科</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>350.4332027292168</v>
+        <v>353.0156864752025</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>91.90000000000001</v>
+        <v>65.2</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,13 +3467,13 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>49.83579386842955</v>
+        <v>49.27097146593565</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>15.31391985134478</v>
+        <v>11.07449581396929</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.7851852545223736</v>
+        <v>0.8157288007792904</v>
       </c>
       <c r="K57" s="2" t="n">
         <v>0</v>
@@ -3485,31 +3485,31 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>1.517309099665173</v>
+        <v>0.7405550201103304</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>8080</v>
+        <v>8150</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>永利聯合</t>
+          <t>南茂</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>342.1073850928092</v>
+        <v>350.4332027292168</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>28.05</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,13 +3520,13 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>51.19058610380378</v>
+        <v>49.83579386842955</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>47.03556838832704</v>
+        <v>15.31391985134478</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>0.4924843126333495</v>
+        <v>0.7851852545223736</v>
       </c>
       <c r="K58" s="2" t="n">
         <v>0</v>
@@ -3538,31 +3538,31 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.026998375032521</v>
+        <v>1.517309099665173</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>8091</v>
+        <v>8080</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>翔名</t>
+          <t>永利聯合</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>339.5981800412615</v>
+        <v>342.1073850928092</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>230</v>
+        <v>28.05</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,13 +3573,13 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>45.95755479965909</v>
+        <v>51.19058610380378</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>13.09569640157622</v>
+        <v>47.03556838832704</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.5086757917273701</v>
+        <v>0.4924843126333495</v>
       </c>
       <c r="K59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>1.999481198655985</v>
+        <v>0.026998375032521</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>8213</v>
+        <v>8091</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>志超</t>
+          <t>翔名</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>332.1708598539261</v>
+        <v>339.5981800412615</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>33</v>
+        <v>230</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,13 +3626,13 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>55.50665767470076</v>
+        <v>45.95755479965909</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>28.60911042801965</v>
+        <v>13.09569640157622</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>0.6912317470033642</v>
+        <v>0.5086757917273701</v>
       </c>
       <c r="K60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.5896158985190484</v>
+        <v>1.999481198655985</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, adx_trending, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>8050</v>
+        <v>8213</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>廣積</t>
+          <t>志超</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>330.7069026016333</v>
+        <v>332.1708598539261</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>58</v>
+        <v>33</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,13 +3679,13 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>47.07038415856739</v>
+        <v>55.50665767470076</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>19.13216262757745</v>
+        <v>28.60911042801965</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>0.4706902601633332</v>
+        <v>0.6912317470033642</v>
       </c>
       <c r="K61" s="2" t="n">
         <v>0</v>
@@ -3697,31 +3697,31 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-0.4685567513680959</v>
+        <v>0.5896158985190484</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, above_ichimoku_cloud</t>
+          <t>rsi_strong, market_above_ma60, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>9930</v>
+        <v>8050</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>中聯資源</t>
+          <t>廣積</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>317.2770725758377</v>
+        <v>330.7069026016333</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>62.8</v>
+        <v>58</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3732,13 +3732,13 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>42.10828412104235</v>
+        <v>47.07038415856739</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>44.86181174810068</v>
+        <v>19.13216262757745</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>0.6236744838134081</v>
+        <v>0.4706902601633332</v>
       </c>
       <c r="K62" s="2" t="n">
         <v>0</v>
@@ -3750,31 +3750,31 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>0.1290994160141183</v>
+        <v>-0.4685567513680959</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>8454</v>
+        <v>9930</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>富邦媒</t>
+          <t>中聯資源</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>315.9559288420491</v>
+        <v>317.2770725758377</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>262.5</v>
+        <v>62.8</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,13 +3785,13 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>48.80806781583413</v>
+        <v>42.10828412104235</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>16.94822637430592</v>
+        <v>44.86181174810068</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>0.4216395011907233</v>
+        <v>0.6236744838134081</v>
       </c>
       <c r="K63" s="2" t="n">
         <v>0</v>
@@ -3803,31 +3803,31 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>2.963739803443314</v>
+        <v>0.1290994160141183</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>8163</v>
+        <v>8454</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>達方</t>
+          <t>富邦媒</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>312.5770361021542</v>
+        <v>315.9559288420491</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>31.95</v>
+        <v>262.5</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3838,13 +3838,13 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>44.10097613061173</v>
+        <v>48.80806781583413</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>22.92261101388632</v>
+        <v>16.94822637430592</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>0.4611456653765202</v>
+        <v>0.4216395011907233</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>0</v>
@@ -3856,31 +3856,31 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>0.4478079323226394</v>
+        <v>2.963739803443314</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>8086</v>
+        <v>8163</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>宏捷科</t>
+          <t>達方</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>311.811147305081</v>
+        <v>312.5770361021542</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>114</v>
+        <v>31.95</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3891,13 +3891,13 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>42.46936875675626</v>
+        <v>44.10097613061173</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>26.77931346500181</v>
+        <v>22.92261101388632</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.7006678952102374</v>
+        <v>0.4611456653765202</v>
       </c>
       <c r="K65" s="2" t="n">
         <v>0</v>
@@ -3909,31 +3909,31 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>1.207336518270437</v>
+        <v>0.4478079323226394</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>8183</v>
+        <v>8086</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>精星</t>
+          <t>宏捷科</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>308.1971701424783</v>
+        <v>311.811147305081</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>30.05</v>
+        <v>114</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3944,13 +3944,13 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>47.25433089970152</v>
+        <v>42.46936875675626</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>21.73603246961148</v>
+        <v>26.77931346500181</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>0.9703860471276112</v>
+        <v>0.7006678952102374</v>
       </c>
       <c r="K66" s="2" t="n">
         <v>0</v>
@@ -3962,31 +3962,31 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>0.2501116501726539</v>
+        <v>1.207336518270437</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>8048</v>
+        <v>8183</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>德勝</t>
+          <t>精星</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>300.4868817354571</v>
+        <v>308.1971701424783</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>51.5</v>
+        <v>30.05</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3997,13 +3997,13 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>39.91842464313299</v>
+        <v>47.25433089970152</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>19.36114633977246</v>
+        <v>21.73603246961148</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.3872745909597485</v>
+        <v>0.9703860471276112</v>
       </c>
       <c r="K67" s="2" t="n">
         <v>0</v>
@@ -4015,31 +4015,31 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.347645971725762</v>
+        <v>0.2501116501726539</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>8047</v>
+        <v>8048</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>星雲</t>
+          <t>德勝</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>299.720043622505</v>
+        <v>300.4868817354571</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>45.1</v>
+        <v>51.5</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -4050,13 +4050,13 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>49.61906990449541</v>
+        <v>39.91842464313299</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>11.80320053759852</v>
+        <v>19.36114633977246</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>0.9402815611552138</v>
+        <v>0.3872745909597485</v>
       </c>
       <c r="K68" s="2" t="n">
         <v>0</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>0.2976931537436278</v>
+        <v>0.347645971725762</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4078,21 +4078,21 @@
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>8374</v>
+        <v>8047</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>羅昇</t>
+          <t>星雲</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>297.8127781087577</v>
+        <v>299.720043622505</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>85.7</v>
+        <v>45.1</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -4103,13 +4103,13 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>55.45601856990545</v>
+        <v>49.61906990449541</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>19.78656421992343</v>
+        <v>11.80320053759852</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>1.205599955135406</v>
+        <v>0.9402815611552138</v>
       </c>
       <c r="K69" s="2" t="n">
         <v>0</v>
@@ -4121,31 +4121,31 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>1.778771622343975</v>
+        <v>0.2976931537436278</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>8059</v>
+        <v>8374</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>凱碩</t>
+          <t>羅昇</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>297.3940251537916</v>
+        <v>297.8127781087577</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>14.1</v>
+        <v>85.7</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,13 +4156,13 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>33.86949824704377</v>
+        <v>55.45601856990545</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>22.93305256991027</v>
+        <v>19.78656421992343</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>3.363496388290458</v>
+        <v>1.205599955135406</v>
       </c>
       <c r="K70" s="2" t="n">
         <v>0</v>
@@ -4174,31 +4174,31 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.023632837467423</v>
+        <v>1.778771622343975</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>rsi_strong, market_above_ma60, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>8054</v>
+        <v>8059</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>安國</t>
+          <t>凱碩</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>296.2492476382554</v>
+        <v>297.3940251537916</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>82.59999999999999</v>
+        <v>14.1</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,13 +4209,13 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>39.25544681450984</v>
+        <v>33.86949824704377</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>20.73168815495861</v>
+        <v>22.93305256991027</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>0.7912604691473574</v>
+        <v>3.363496388290458</v>
       </c>
       <c r="K71" s="2" t="n">
         <v>0</v>
@@ -4227,31 +4227,31 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.8912507531641571</v>
+        <v>0.023632837467423</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>8101</v>
+        <v>8054</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>華冠</t>
+          <t>安國</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>290.1265996849627</v>
+        <v>296.2492476382554</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>11.5</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,13 +4262,13 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>50.10776216767238</v>
+        <v>39.25544681450984</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>13.26199516287776</v>
+        <v>20.73168815495861</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>1.594597816645946</v>
+        <v>0.7912604691473574</v>
       </c>
       <c r="K72" s="2" t="n">
         <v>0</v>
@@ -4280,31 +4280,31 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>0.2073077613873822</v>
+        <v>0.8912507531641571</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>8064</v>
+        <v>8101</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>東捷</t>
+          <t>華冠</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>285.3351841699936</v>
+        <v>290.1265996849627</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>102.5</v>
+        <v>11.5</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -4315,16 +4315,16 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>43.36345889274169</v>
+        <v>50.10776216767238</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>20.45295983911442</v>
+        <v>13.26199516287776</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>0.5620008437960001</v>
+        <v>1.594597816645946</v>
       </c>
       <c r="K73" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L73" s="2" t="n">
         <v>0</v>
@@ -4333,31 +4333,31 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>1.890934189528685</v>
+        <v>0.2073077613873822</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>volume_break, market_above_ma60, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>8932</v>
+        <v>8064</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>智通*</t>
+          <t>東捷</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>283.5934981542632</v>
+        <v>285.3351841699936</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>108</v>
+        <v>102.5</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,13 +4368,13 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>53.75733401813656</v>
+        <v>43.36345889274169</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>16.69583301976951</v>
+        <v>20.45295983911442</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.8072779613834299</v>
+        <v>0.5620008437960001</v>
       </c>
       <c r="K74" s="2" t="n">
         <v>1</v>
@@ -4386,31 +4386,31 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>1.02743671899334</v>
+        <v>1.890934189528685</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>8044</v>
+        <v>8932</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>網家</t>
+          <t>智通*</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>280.5882763151578</v>
+        <v>283.5934981542632</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>26.45</v>
+        <v>108</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4421,16 +4421,16 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>45.34874076538357</v>
+        <v>53.75733401813656</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>13.22190646460483</v>
+        <v>16.69583301976951</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>0.5087502513112772</v>
+        <v>0.8072779613834299</v>
       </c>
       <c r="K75" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L75" s="2" t="n">
         <v>0</v>
@@ -4439,31 +4439,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>0.06554175310208681</v>
+        <v>1.02743671899334</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>8103</v>
+        <v>8044</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>瀚荃</t>
+          <t>網家</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>279.091004939701</v>
+        <v>280.5882763151578</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>78.90000000000001</v>
+        <v>26.45</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,13 +4474,13 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>45.52544774695405</v>
+        <v>45.34874076538357</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>24.47110978610414</v>
+        <v>13.22190646460483</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>0.7857498455720749</v>
+        <v>0.5087502513112772</v>
       </c>
       <c r="K76" s="2" t="n">
         <v>0</v>
@@ -4492,31 +4492,31 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>1.300686818685819</v>
+        <v>0.06554175310208681</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>8455</v>
+        <v>8103</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>大拓-KY</t>
+          <t>瀚荃</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>277.6862267133371</v>
+        <v>279.091004939701</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>26</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,13 +4527,13 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>51.71191941769705</v>
+        <v>45.52544774695405</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>15.47780414524021</v>
+        <v>24.47110978610414</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>1.710007770870338</v>
+        <v>0.7857498455720749</v>
       </c>
       <c r="K77" s="2" t="n">
         <v>0</v>
@@ -4545,31 +4545,31 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>0.325301260201448</v>
+        <v>1.300686818685819</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>8114</v>
+        <v>8455</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>振樺電</t>
+          <t>大拓-KY</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>266.0308917528171</v>
+        <v>277.6862267133371</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>204</v>
+        <v>26</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4580,13 +4580,13 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>45.5035248194376</v>
+        <v>51.71191941769705</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>13.81313475112184</v>
+        <v>15.47780414524021</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>0.4930668721725793</v>
+        <v>1.710007770870338</v>
       </c>
       <c r="K78" s="2" t="n">
         <v>0</v>
@@ -4598,31 +4598,31 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.9532305320153708</v>
+        <v>0.325301260201448</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>8472</v>
+        <v>8114</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>夠麻吉</t>
+          <t>振樺電</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>265.3917282453597</v>
+        <v>266.0308917528171</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>69.2</v>
+        <v>204</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4633,16 +4633,16 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>41.12750081258253</v>
+        <v>45.5035248194376</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>16.07890371333362</v>
+        <v>13.81313475112184</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>0.4683760251728103</v>
+        <v>0.4930668721725793</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L79" s="2" t="n">
         <v>0</v>
@@ -4651,31 +4651,31 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>0.5270456911613364</v>
+        <v>-0.9532305320153708</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>8147</v>
+        <v>8472</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>正淩</t>
+          <t>夠麻吉</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>253.3219723221557</v>
+        <v>265.3917282453597</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>121</v>
+        <v>69.2</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4686,16 +4686,16 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>41.5913681101342</v>
+        <v>41.12750081258253</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>27.42109552250149</v>
+        <v>16.07890371333362</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>1.153541539219854</v>
+        <v>0.4683760251728103</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L80" s="2" t="n">
         <v>0</v>
@@ -4704,31 +4704,31 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>1.553764880352757</v>
+        <v>0.5270456911613364</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>8440</v>
+        <v>8147</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>綠電</t>
+          <t>正淩</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>249.0677594378676</v>
+        <v>253.3219723221557</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>20.1</v>
+        <v>121</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4739,13 +4739,13 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>50.88965138830331</v>
+        <v>41.5913681101342</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>18.85451076989961</v>
+        <v>27.42109552250149</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>1.345303160685629</v>
+        <v>1.153541539219854</v>
       </c>
       <c r="K81" s="2" t="n">
         <v>0</v>
@@ -4757,31 +4757,31 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.1812445436482078</v>
+        <v>1.553764880352757</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>8104</v>
+        <v>8440</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>錸寶</t>
+          <t>綠電</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>247.7792012364933</v>
+        <v>249.0677594378676</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>31.85</v>
+        <v>20.1</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4792,13 +4792,13 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>43.43161999121229</v>
+        <v>50.88965138830331</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>29.05563583213562</v>
+        <v>18.85451076989961</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>0.7592036527001075</v>
+        <v>1.345303160685629</v>
       </c>
       <c r="K82" s="2" t="n">
         <v>0</v>
@@ -4810,31 +4810,31 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>0.3804632219717452</v>
+        <v>0.1812445436482078</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>8176</v>
+        <v>8104</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>智捷</t>
+          <t>錸寶</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>245.5383649094016</v>
+        <v>247.7792012364933</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>10.1</v>
+        <v>31.85</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4845,13 +4845,13 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>53.69259191870899</v>
+        <v>43.43161999121229</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>12.728683906165</v>
+        <v>29.05563583213562</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>1.170332225234253</v>
+        <v>0.7592036527001075</v>
       </c>
       <c r="K83" s="2" t="n">
         <v>0</v>
@@ -4863,31 +4863,31 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.0426940351263855</v>
+        <v>0.3804632219717452</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>8478</v>
+        <v>8176</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>東哥遊艇</t>
+          <t>智捷</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>245.3986683610383</v>
+        <v>245.5383649094016</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>143.5</v>
+        <v>10.1</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4898,13 +4898,13 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>33.54451342471457</v>
+        <v>53.69259191870899</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>8.760176306646258</v>
+        <v>12.728683906165</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>1.651315988892332</v>
+        <v>1.170332225234253</v>
       </c>
       <c r="K84" s="2" t="n">
         <v>0</v>
@@ -4916,31 +4916,31 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.5853016046147816</v>
+        <v>0.0426940351263855</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>9136</v>
+        <v>8478</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>巨騰-DR</t>
+          <t>東哥遊艇</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>241.3548365832253</v>
+        <v>245.3986683610383</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>11.5</v>
+        <v>143.5</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4951,13 +4951,13 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>45.54405106946568</v>
+        <v>33.54451342471457</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>10.49675326612626</v>
+        <v>8.760176306646258</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.774578886336485</v>
+        <v>1.651315988892332</v>
       </c>
       <c r="K85" s="2" t="n">
         <v>0</v>
@@ -4969,31 +4969,31 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>0.09978306923721871</v>
+        <v>-0.5853016046147816</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>8291</v>
+        <v>9136</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>尚茂</t>
+          <t>巨騰-DR</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>240.5959840959474</v>
+        <v>241.3548365832253</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>35</v>
+        <v>11.5</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5004,13 +5004,13 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>42.70047967921641</v>
+        <v>45.54405106946568</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>12.88397460260428</v>
+        <v>10.49675326612626</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>0.5132583938060374</v>
+        <v>0.774578886336485</v>
       </c>
       <c r="K86" s="2" t="n">
         <v>0</v>
@@ -5022,31 +5022,31 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>0.1265539949361254</v>
+        <v>0.09978306923721871</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>8201</v>
+        <v>8291</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>無敵</t>
+          <t>尚茂</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>238.016263332268</v>
+        <v>240.5959840959474</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>11.85</v>
+        <v>35</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5057,13 +5057,13 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>42.21474602363968</v>
+        <v>42.70047967921641</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>23.1355704684553</v>
+        <v>12.88397460260428</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>0.2767528939173276</v>
+        <v>0.5132583938060374</v>
       </c>
       <c r="K87" s="2" t="n">
         <v>0</v>
@@ -5075,31 +5075,31 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.0633154703912594</v>
+        <v>0.1265539949361254</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>8068</v>
+        <v>8201</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>全達</t>
+          <t>無敵</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>236.1593824764996</v>
+        <v>238.016263332268</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>17.6</v>
+        <v>11.85</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>44.3080673302498</v>
+        <v>42.21474602363968</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>12.85634028930056</v>
+        <v>23.1355704684553</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>0.4341072039516288</v>
+        <v>0.2767528939173276</v>
       </c>
       <c r="K88" s="2" t="n">
         <v>0</v>
@@ -5128,31 +5128,31 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.0623132388782099</v>
+        <v>0.0633154703912594</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>8087</v>
+        <v>8068</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>華鎂鑫</t>
+          <t>全達</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>235.4679928557301</v>
+        <v>236.1593824764996</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>26.55</v>
+        <v>17.6</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,13 +5163,13 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>49.9876239806284</v>
+        <v>44.3080673302498</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>14.10218119928922</v>
+        <v>12.85634028930056</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>1.853384256312328</v>
+        <v>0.4341072039516288</v>
       </c>
       <c r="K89" s="2" t="n">
         <v>0</v>
@@ -5181,31 +5181,31 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>0.9708285937277999</v>
+        <v>0.0623132388782099</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>8076</v>
+        <v>8087</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>伍豐</t>
+          <t>華鎂鑫</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>235.2304621765166</v>
+        <v>235.4679928557301</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>23.6</v>
+        <v>26.55</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -5216,13 +5216,13 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>49.06885661733421</v>
+        <v>49.9876239806284</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>10.87889349477208</v>
+        <v>14.10218119928922</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>0.5680403311738006</v>
+        <v>1.853384256312328</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>0</v>
@@ -5234,31 +5234,31 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.1711668547250383</v>
+        <v>0.9708285937277999</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>9110</v>
+        <v>8076</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>越南控-DR</t>
+          <t>伍豐</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>234.0382038737484</v>
+        <v>235.2304621765166</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>3.11</v>
+        <v>23.6</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5269,13 +5269,13 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>51.60825187961324</v>
+        <v>49.06885661733421</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>7.607874557679624</v>
+        <v>10.87889349477208</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>0.6574049904772954</v>
+        <v>0.5680403311738006</v>
       </c>
       <c r="K91" s="2" t="n">
         <v>0</v>
@@ -5287,31 +5287,31 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>0.0244353882153277</v>
+        <v>0.1711668547250383</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>8171</v>
+        <v>9110</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>天宇</t>
+          <t>越南控-DR</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>232.6957352459142</v>
+        <v>234.0382038737484</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>19.7</v>
+        <v>3.11</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5322,13 +5322,13 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>43.38518095461364</v>
+        <v>51.60825187961324</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>14.3510297427896</v>
+        <v>7.607874557679624</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>1.893067323084326</v>
+        <v>0.6574049904772954</v>
       </c>
       <c r="K92" s="2" t="n">
         <v>0</v>
@@ -5340,31 +5340,31 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>0.1285403184872928</v>
+        <v>0.0244353882153277</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>8499</v>
+        <v>8171</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>鼎炫-KY</t>
+          <t>天宇</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>231.5264195332832</v>
+        <v>232.6957352459142</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>262</v>
+        <v>19.7</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,13 +5375,13 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>47.57695838439179</v>
+        <v>43.38518095461364</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>19.47003333583104</v>
+        <v>14.3510297427896</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>0.5696696370146953</v>
+        <v>1.893067323084326</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>0</v>
@@ -5393,31 +5393,31 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>3.118761614444166</v>
+        <v>0.1285403184872928</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>9103</v>
+        <v>8499</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>美德醫療-DR</t>
+          <t>鼎炫-KY</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>230.3066824644803</v>
+        <v>231.5264195332832</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>5.16</v>
+        <v>262</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5428,13 +5428,13 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>47.67513060704312</v>
+        <v>47.57695838439179</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>16.8251619104483</v>
+        <v>19.47003333583104</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>0.5153390088081791</v>
+        <v>0.5696696370146953</v>
       </c>
       <c r="K94" s="2" t="n">
         <v>0</v>
@@ -5446,31 +5446,31 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-0.0060992943405242</v>
+        <v>3.118761614444166</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>8442</v>
+        <v>9103</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>威宏-KY</t>
+          <t>美德醫療-DR</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>221.9463746571386</v>
+        <v>230.3066824644803</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>43.7</v>
+        <v>5.16</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5481,13 +5481,13 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>46.60807079025937</v>
+        <v>47.67513060704312</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>20.70412706008145</v>
+        <v>16.8251619104483</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>0.3554198125035117</v>
+        <v>0.5153390088081791</v>
       </c>
       <c r="K95" s="2" t="n">
         <v>0</v>
@@ -5499,31 +5499,31 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.1819499753038357</v>
+        <v>-0.0060992943405242</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>8071</v>
+        <v>8442</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>能率網通</t>
+          <t>威宏-KY</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>220.5161193130371</v>
+        <v>221.9463746571386</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>24.4</v>
+        <v>43.7</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,13 +5534,13 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>50.54491831462373</v>
+        <v>46.60807079025937</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>18.65049008900301</v>
+        <v>20.70412706008145</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.7599320386264472</v>
+        <v>0.3554198125035117</v>
       </c>
       <c r="K96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.4141175502683568</v>
+        <v>-0.1819499753038357</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>9802</v>
+        <v>8071</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>鈺齊-KY</t>
+          <t>能率網通</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>219.30167297669</v>
+        <v>220.5161193130371</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>71.59999999999999</v>
+        <v>24.4</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,13 +5587,13 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>46.24264608299816</v>
+        <v>50.54491831462373</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>13.6437546420352</v>
+        <v>18.65049008900301</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.8147811788519328</v>
+        <v>0.7599320386264472</v>
       </c>
       <c r="K97" s="2" t="n">
         <v>0</v>
@@ -5605,31 +5605,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>0.2189549551341082</v>
+        <v>0.4141175502683568</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>8477</v>
+        <v>9802</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>創業家</t>
+          <t>鈺齊-KY</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>201.5610123147142</v>
+        <v>219.30167297669</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>15.95</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,13 +5640,13 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>51.64701521087193</v>
+        <v>46.24264608299816</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>7.785016749395396</v>
+        <v>13.6437546420352</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>1.210818625945891</v>
+        <v>0.8147811788519328</v>
       </c>
       <c r="K98" s="2" t="n">
         <v>0</v>
@@ -5658,31 +5658,31 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>0.1902771267297427</v>
+        <v>0.2189549551341082</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>8481</v>
+        <v>8477</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>政伸</t>
+          <t>創業家</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>196.2353762987931</v>
+        <v>201.5610123147142</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>41</v>
+        <v>15.95</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,13 +5693,13 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>52.8096071226651</v>
+        <v>51.64701521087193</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>17.44856976219705</v>
+        <v>7.785016749395396</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.2098675593072333</v>
+        <v>1.210818625945891</v>
       </c>
       <c r="K99" s="2" t="n">
         <v>0</v>
@@ -5711,31 +5711,31 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>0.1402512608453791</v>
+        <v>0.1902771267297427</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>8466</v>
+        <v>8481</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>美吉吉-KY</t>
+          <t>政伸</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>195.5105983026336</v>
+        <v>196.2353762987931</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>16.1</v>
+        <v>41</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,13 +5746,13 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>38.79063620601213</v>
+        <v>52.8096071226651</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>21.19951490941506</v>
+        <v>17.44856976219705</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>0.9473110984969104</v>
+        <v>0.2098675593072333</v>
       </c>
       <c r="K100" s="2" t="n">
         <v>0</v>
@@ -5764,31 +5764,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.1110500526128818</v>
+        <v>0.1402512608453791</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>9902</v>
+        <v>8466</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>台火</t>
+          <t>美吉吉-KY</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>193.3947838651259</v>
+        <v>195.5105983026336</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>13.7</v>
+        <v>16.1</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,13 +5799,13 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>48.72123189382678</v>
+        <v>38.79063620601213</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>10.24662944486864</v>
+        <v>21.19951490941506</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>0.8630397916783874</v>
+        <v>0.9473110984969104</v>
       </c>
       <c r="K101" s="2" t="n">
         <v>0</v>
@@ -5817,31 +5817,31 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>0.0185587764496632</v>
+        <v>-0.1110500526128818</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>8277</v>
+        <v>9902</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>商丞</t>
+          <t>台火</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>187.553525392494</v>
+        <v>193.3947838651259</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>8.109999999999999</v>
+        <v>13.7</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,16 +5852,16 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>45.18339306820933</v>
+        <v>48.72123189382678</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>14.1774150237132</v>
+        <v>10.24662944486864</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>0.3562813440781449</v>
+        <v>0.8630397916783874</v>
       </c>
       <c r="K102" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L102" s="2" t="n">
         <v>0</v>
@@ -5870,31 +5870,31 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>0.0627955340569044</v>
+        <v>0.0185587764496632</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>8072</v>
+        <v>8277</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>陞泰</t>
+          <t>商丞</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>181.3022651795711</v>
+        <v>187.553525392494</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>26.55</v>
+        <v>8.109999999999999</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,16 +5905,16 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>45.47627659370166</v>
+        <v>45.18339306820933</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>19.40022568163664</v>
+        <v>14.1774150237132</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>0.4942643056517879</v>
+        <v>0.3562813440781449</v>
       </c>
       <c r="K103" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L103" s="2" t="n">
         <v>0</v>
@@ -5923,31 +5923,31 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>0.08410668690876789</v>
+        <v>0.0627955340569044</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>8467</v>
+        <v>8072</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>波力-KY</t>
+          <t>陞泰</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>179.4017184016702</v>
+        <v>181.3022651795711</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>101.5</v>
+        <v>26.55</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,13 +5958,13 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>45.48773252062031</v>
+        <v>45.47627659370166</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>14.70480369055645</v>
+        <v>19.40022568163664</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>0.9645439701422908</v>
+        <v>0.4942643056517879</v>
       </c>
       <c r="K104" s="2" t="n">
         <v>0</v>
@@ -5976,31 +5976,31 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>1.004763368722426</v>
+        <v>0.08410668690876789</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>8423</v>
+        <v>8467</v>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>保綠-KY</t>
+          <t>波力-KY</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>173.953753271435</v>
+        <v>179.4017184016702</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>17.8</v>
+        <v>101.5</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -6011,16 +6011,16 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>50.68912026598469</v>
+        <v>45.48773252062031</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>18.82670288870662</v>
+        <v>14.70480369055645</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>0.310466640769156</v>
+        <v>0.9645439701422908</v>
       </c>
       <c r="K105" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L105" s="2" t="n">
         <v>0</v>
@@ -6029,31 +6029,31 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>0.0073593481576178</v>
+        <v>1.004763368722426</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>8410</v>
+        <v>8423</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>森田</t>
+          <t>保綠-KY</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>173.184073265946</v>
+        <v>173.953753271435</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>31.9</v>
+        <v>17.8</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -6064,16 +6064,16 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>51.73880197305544</v>
+        <v>50.68912026598469</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>23.43469945819869</v>
+        <v>18.82670288870662</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>0.8654061327946674</v>
+        <v>0.310466640769156</v>
       </c>
       <c r="K106" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L106" s="2" t="n">
         <v>0</v>
@@ -6082,31 +6082,31 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.2109880889877383</v>
+        <v>0.0073593481576178</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>8404</v>
+        <v>8410</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>百和興業-KY</t>
+          <t>森田</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>167.7762567487448</v>
+        <v>173.184073265946</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>16.1</v>
+        <v>31.9</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -6117,13 +6117,13 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>37.86831162247513</v>
+        <v>51.73880197305544</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>17.86955730364468</v>
+        <v>23.43469945819869</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>1.271698984203642</v>
+        <v>0.8654061327946674</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>0</v>
@@ -6135,31 +6135,31 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-0.0287700704564866</v>
+        <v>0.2109880889877383</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>8341</v>
+        <v>8404</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>日友</t>
+          <t>百和興業-KY</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>162.1772104898174</v>
+        <v>167.7762567487448</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>75.90000000000001</v>
+        <v>16.1</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -6170,13 +6170,13 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>46.35460714005259</v>
+        <v>37.86831162247513</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>10.89813184544015</v>
+        <v>17.86955730364468</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>0.7972948932789204</v>
+        <v>1.271698984203642</v>
       </c>
       <c r="K108" s="2" t="n">
         <v>0</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>0.0798362269747131</v>
+        <v>-0.0287700704564866</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6198,21 +6198,21 @@
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>8097</v>
+        <v>8341</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>常珵</t>
+          <t>日友</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>159.0936093690173</v>
+        <v>162.1772104898174</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>50.6</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,13 +6223,13 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>34.2607942057747</v>
+        <v>46.35460714005259</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>15.8012119670854</v>
+        <v>10.89813184544015</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>0.8270218984131174</v>
+        <v>0.7972948932789204</v>
       </c>
       <c r="K109" s="2" t="n">
         <v>0</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.0585132603350253</v>
+        <v>0.0798362269747131</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6251,21 +6251,21 @@
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>8482</v>
+        <v>8097</v>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>商億-KY</t>
+          <t>常珵</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>152.1236243486709</v>
+        <v>159.0936093690173</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>47.75</v>
+        <v>50.6</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
@@ -6276,13 +6276,13 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>50.86784088693</v>
+        <v>34.2607942057747</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>5.009272730518751</v>
+        <v>15.8012119670854</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>0.3028226144851316</v>
+        <v>0.8270218984131174</v>
       </c>
       <c r="K110" s="2" t="n">
         <v>0</v>
@@ -6294,31 +6294,31 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>0.2728388099976389</v>
+        <v>0.0585132603350253</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>8089</v>
+        <v>8482</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>康全電訊</t>
+          <t>商億-KY</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>142.8427316928839</v>
+        <v>152.1236243486709</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>17.9</v>
+        <v>47.75</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -6329,13 +6329,13 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>40.44023349908021</v>
+        <v>50.86784088693</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>11.91498439360699</v>
+        <v>5.009272730518751</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>0.623020281272849</v>
+        <v>0.3028226144851316</v>
       </c>
       <c r="K111" s="2" t="n">
         <v>0</v>
@@ -6347,31 +6347,31 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>0.006896205615666</v>
+        <v>0.2728388099976389</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>8431</v>
+        <v>8089</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>匯鑽科</t>
+          <t>康全電訊</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>141.0192545327979</v>
+        <v>142.8427316928839</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>47.8</v>
+        <v>17.9</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -6382,16 +6382,16 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>46.08118863974775</v>
+        <v>40.44023349908021</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>13.17695418465223</v>
+        <v>11.91498439360699</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>0.5251872760037121</v>
+        <v>0.623020281272849</v>
       </c>
       <c r="K112" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L112" s="2" t="n">
         <v>0</v>
@@ -6400,31 +6400,31 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.2380239075060303</v>
+        <v>0.006896205615666</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>8487</v>
+        <v>8431</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>愛爾達-創</t>
+          <t>匯鑽科</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>136.8696902145726</v>
+        <v>141.0192545327979</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>72.2</v>
+        <v>47.8</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6435,16 +6435,16 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>31.60972465889192</v>
+        <v>46.08118863974775</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>18.91270352736331</v>
+        <v>13.17695418465223</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>0.3383874187736268</v>
+        <v>0.5251872760037121</v>
       </c>
       <c r="K113" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L113" s="2" t="n">
         <v>0</v>
@@ -6453,31 +6453,31 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.1200600700558072</v>
+        <v>0.2380239075060303</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>8085</v>
+        <v>8487</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>福華</t>
+          <t>愛爾達-創</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>125.3121070422506</v>
+        <v>136.8696902145726</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>11.25</v>
+        <v>72.2</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,13 +6488,13 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>45.13709686029026</v>
+        <v>31.60972465889192</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>10.44860893685265</v>
+        <v>18.91270352736331</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>0.3317832667978202</v>
+        <v>0.3383874187736268</v>
       </c>
       <c r="K114" s="2" t="n">
         <v>0</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>0.0410958795899379</v>
+        <v>-0.1200600700558072</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6516,21 +6516,21 @@
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>8476</v>
+        <v>8085</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>台境*</t>
+          <t>福華</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>120.7035486190409</v>
+        <v>125.3121070422506</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>20.1</v>
+        <v>11.25</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,13 +6541,13 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>43.22718186769026</v>
+        <v>45.13709686029026</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>17.58041564244024</v>
+        <v>10.44860893685265</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>0.2601412456714305</v>
+        <v>0.3317832667978202</v>
       </c>
       <c r="K115" s="2" t="n">
         <v>0</v>
@@ -6559,31 +6559,31 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.08407440591090951</v>
+        <v>0.0410958795899379</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
-        <v>8045</v>
+        <v>8476</v>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>達運光電</t>
+          <t>台境*</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>111.4428112240852</v>
+        <v>120.7035486190409</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>50.8</v>
+        <v>20.1</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
@@ -6594,13 +6594,13 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>37.86549392490329</v>
+        <v>43.22718186769026</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>19.72952116093148</v>
+        <v>17.58041564244024</v>
       </c>
       <c r="J116" s="2" t="n">
-        <v>0.6629389660603151</v>
+        <v>0.2601412456714305</v>
       </c>
       <c r="K116" s="2" t="n">
         <v>0</v>
@@ -6612,62 +6612,115 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.281362040952787</v>
+        <v>-0.08407440591090951</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
+        <v>8045</v>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>達運光電</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D117" s="2" t="n">
+        <v>111.4428112240852</v>
+      </c>
+      <c r="E117" s="2" t="n">
+        <v>50.8</v>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="G117" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H117" s="2" t="n">
+        <v>37.86549392490329</v>
+      </c>
+      <c r="I117" s="2" t="n">
+        <v>19.72952116093148</v>
+      </c>
+      <c r="J117" s="2" t="n">
+        <v>0.6629389660603151</v>
+      </c>
+      <c r="K117" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L117" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M117" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N117" s="2" t="n">
+        <v>-0.281362040952787</v>
+      </c>
+      <c r="O117" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="n">
         <v>8092</v>
       </c>
-      <c r="B117" s="2" t="inlineStr">
+      <c r="B118" s="2" t="inlineStr">
         <is>
           <t>建暐</t>
         </is>
       </c>
-      <c r="C117" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D117" s="2" t="n">
+      <c r="C118" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D118" s="2" t="n">
         <v>107.0375243086058</v>
       </c>
-      <c r="E117" s="2" t="n">
+      <c r="E118" s="2" t="n">
         <v>12.5</v>
       </c>
-      <c r="F117" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="G117" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H117" s="2" t="n">
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="G118" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H118" s="2" t="n">
         <v>33.75027091502308</v>
       </c>
-      <c r="I117" s="2" t="n">
+      <c r="I118" s="2" t="n">
         <v>19.02286827345237</v>
       </c>
-      <c r="J117" s="2" t="n">
+      <c r="J118" s="2" t="n">
         <v>0.892730443969816</v>
       </c>
-      <c r="K117" s="2" t="n">
+      <c r="K118" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L117" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M117" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N117" s="2" t="n">
+      <c r="L118" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M118" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N118" s="2" t="n">
         <v>-0.0304818403175157</v>
       </c>
-      <c r="O117" s="2" t="inlineStr">
+      <c r="O118" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, avoid_chase</t>
         </is>

</xml_diff>